<commit_message>
WM 2026 Prognose: Datum und Spieltag je Begegnung ergaenzt (Excel + Markdown)
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -490,14 +490,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,20 +524,30 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Spieltag</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>Begegnung</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Sieger-Tipp</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Ergebnis-Tipp</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Wertigkeit</t>
         </is>
@@ -547,22 +559,30 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>11.06.2026</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Mexiko - Suedafrika</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Mexiko (gespielt)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -574,22 +594,30 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>11.06.2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Suedkorea - Tschechien</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Suedkorea (gespielt)</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -601,22 +629,30 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>18.06.2026</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Mexiko - Suedkorea</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Mexiko</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="G7" s="8" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -626,23 +662,31 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Mexiko - Tschechien</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Mexiko</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>0.6</v>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>18.06.2026</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Tschechien - Suedafrika</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Tschechien</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>0.55</v>
       </c>
     </row>
     <row r="9">
@@ -651,23 +695,31 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Suedkorea - Suedafrika</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Suedkorea</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>24.06.2026</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Mexiko - Tschechien</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Mexiko</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E9" s="8" t="n">
-        <v>0.65</v>
+      <c r="G9" s="8" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="10">
@@ -676,23 +728,31 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Tschechien - Suedafrika</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Tschechien</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>1:0</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>0.55</v>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>24.06.2026</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Suedkorea - Suedafrika</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Suedkorea</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>0.65</v>
       </c>
     </row>
     <row r="11">
@@ -701,22 +761,30 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>12.06.2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Kanada - Bosnien-Herz.</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Bosnien-Herz. (gespielt)</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>0:5</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -728,22 +796,30 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>13.06.2026</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Katar - Schweiz</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>Schweiz</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="G12" s="8" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -753,22 +829,30 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>18.06.2026</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>Kanada - Katar</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>Kanada</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="G13" s="8" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -778,22 +862,30 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Kanada - Schweiz</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>18.06.2026</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Bosnien-Herz. - Schweiz</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>Schweiz</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="G14" s="8" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -803,23 +895,31 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Bosnien-Herz. - Katar</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Bosnien-Herz.</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>0.62</v>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>24.06.2026</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Kanada - Schweiz</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Schweiz</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="16">
@@ -828,23 +928,31 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Bosnien-Herz. - Schweiz</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Schweiz</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>0.5</v>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>24.06.2026</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Bosnien-Herz. - Katar</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Bosnien-Herz.</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>0.62</v>
       </c>
     </row>
     <row r="17">
@@ -853,22 +961,30 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>13.06.2026</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Brasilien - Marokko</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="G17" s="8" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -878,22 +994,30 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>13.06.2026</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Haiti - Schottland</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>Schottland</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="G18" s="8" t="n">
         <v>0.62</v>
       </c>
     </row>
@@ -903,22 +1027,30 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>19.06.2026</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Brasilien - Haiti</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="G19" s="8" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -928,23 +1060,31 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Brasilien - Schottland</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Brasilien</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="n">
-        <v>0.7</v>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>19.06.2026</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Marokko - Schottland</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>0.55</v>
       </c>
     </row>
     <row r="21">
@@ -953,23 +1093,31 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Marokko - Haiti</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>24.06.2026</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Brasilien - Schottland</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Brasilien</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E21" s="8" t="n">
-        <v>0.75</v>
+      <c r="G21" s="8" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="22">
@@ -978,23 +1126,31 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Marokko - Schottland</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>24.06.2026</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Marokko - Haiti</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>Marokko</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>1:0</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="n">
-        <v>0.55</v>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>0.75</v>
       </c>
     </row>
     <row r="23">
@@ -1003,22 +1159,30 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>12.06.2026</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>USA - Paraguay</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="G23" s="8" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -1028,22 +1192,30 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>13.06.2026</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>Australien - Tuerkei</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>Tuerkei</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E24" s="8" t="n">
+      <c r="G24" s="8" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -1053,22 +1225,30 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>19.06.2026</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>USA - Australien</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E25" s="8" t="n">
+      <c r="G25" s="8" t="n">
         <v>0.62</v>
       </c>
     </row>
@@ -1078,23 +1258,31 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>USA - Tuerkei</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>19.06.2026</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Paraguay - Tuerkei</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>Tuerkei</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E26" s="8" t="n">
-        <v>0.48</v>
+      <c r="G26" s="8" t="n">
+        <v>0.53</v>
       </c>
     </row>
     <row r="27">
@@ -1103,23 +1291,31 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Paraguay - Australien</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>1:0</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="n">
-        <v>0.52</v>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>25.06.2026</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>USA - Tuerkei</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Tuerkei</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>0.48</v>
       </c>
     </row>
     <row r="28">
@@ -1128,23 +1324,31 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Paraguay - Tuerkei</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Tuerkei</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="n">
-        <v>0.53</v>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>25.06.2026</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Paraguay - Australien</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>0.52</v>
       </c>
     </row>
     <row r="29">
@@ -1153,22 +1357,30 @@
           <t>E</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>14.06.2026</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Deutschland - Curacao</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="E29" s="8" t="n">
+      <c r="G29" s="8" t="n">
         <v>0.85</v>
       </c>
     </row>
@@ -1178,22 +1390,30 @@
           <t>E</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>14.06.2026</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Elfenbeinkueste - Ecuador</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="E30" s="7" t="inlineStr">
         <is>
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>0:1</t>
         </is>
       </c>
-      <c r="E30" s="8" t="n">
+      <c r="G30" s="8" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -1203,22 +1423,30 @@
           <t>E</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>20.06.2026</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Deutschland - Elfenbeinkueste</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E31" s="8" t="n">
+      <c r="G31" s="8" t="n">
         <v>0.62</v>
       </c>
     </row>
@@ -1228,23 +1456,31 @@
           <t>E</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Deutschland - Ecuador</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="n">
-        <v>0.58</v>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>20.06.2026</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Curacao - Ecuador</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="n">
+        <v>0.78</v>
       </c>
     </row>
     <row r="33">
@@ -1253,23 +1489,31 @@
           <t>E</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>Curacao - Elfenbeinkueste</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Elfenbeinkueste</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>0:2</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="n">
-        <v>0.75</v>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>25.06.2026</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Deutschland - Ecuador</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>0.58</v>
       </c>
     </row>
     <row r="34">
@@ -1278,23 +1522,31 @@
           <t>E</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>Curacao - Ecuador</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>25.06.2026</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Curacao - Elfenbeinkueste</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Elfenbeinkueste</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="E34" s="8" t="n">
-        <v>0.78</v>
+      <c r="G34" s="8" t="n">
+        <v>0.75</v>
       </c>
     </row>
     <row r="35">
@@ -1303,22 +1555,30 @@
           <t>F</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>14.06.2026</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>Niederlande - Japan</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E35" s="8" t="n">
+      <c r="G35" s="8" t="n">
         <v>0.58</v>
       </c>
     </row>
@@ -1328,22 +1588,30 @@
           <t>F</t>
         </is>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>14.06.2026</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>Schweden - Tunesien</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="E36" s="7" t="inlineStr">
         <is>
           <t>Schweden</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="E36" s="8" t="n">
+      <c r="G36" s="8" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -1353,22 +1621,30 @@
           <t>F</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>20.06.2026</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>Niederlande - Schweden</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E37" s="8" t="n">
+      <c r="G37" s="8" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -1378,23 +1654,31 @@
           <t>F</t>
         </is>
       </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>Niederlande - Tunesien</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>Niederlande</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>20.06.2026</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Japan - Tunesien</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E38" s="8" t="n">
-        <v>0.72</v>
+      <c r="G38" s="8" t="n">
+        <v>0.65</v>
       </c>
     </row>
     <row r="39">
@@ -1403,23 +1687,31 @@
           <t>F</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Japan - Schweden</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="n">
-        <v>0.52</v>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>25.06.2026</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Niederlande - Tunesien</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Niederlande</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>0.72</v>
       </c>
     </row>
     <row r="40">
@@ -1428,23 +1720,31 @@
           <t>F</t>
         </is>
       </c>
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>Japan - Tunesien</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>25.06.2026</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Japan - Schweden</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="n">
-        <v>0.65</v>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="n">
+        <v>0.52</v>
       </c>
     </row>
     <row r="41">
@@ -1453,22 +1753,30 @@
           <t>G</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>15.06.2026</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
         <is>
           <t>Belgien - Aegypten</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>Belgien</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E41" s="8" t="n">
+      <c r="G41" s="8" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -1478,22 +1786,30 @@
           <t>G</t>
         </is>
       </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>15.06.2026</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
         <is>
           <t>Iran - Neuseeland</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="E42" s="7" t="inlineStr">
         <is>
           <t>Iran</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E42" s="8" t="n">
+      <c r="G42" s="8" t="n">
         <v>0.68</v>
       </c>
     </row>
@@ -1503,22 +1819,30 @@
           <t>G</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
         <is>
           <t>Belgien - Iran</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="E43" s="7" t="inlineStr">
         <is>
           <t>Belgien</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E43" s="8" t="n">
+      <c r="G43" s="8" t="n">
         <v>0.62</v>
       </c>
     </row>
@@ -1528,23 +1852,31 @@
           <t>G</t>
         </is>
       </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>Belgien - Neuseeland</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>Belgien</t>
-        </is>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>3:0</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="n">
-        <v>0.82</v>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Aegypten - Neuseeland</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Aegypten</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="45">
@@ -1553,23 +1885,31 @@
           <t>G</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>Aegypten - Iran</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>Aegypten</t>
-        </is>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>1:0</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="n">
-        <v>0.48</v>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>26.06.2026</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Belgien - Neuseeland</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="n">
+        <v>0.82</v>
       </c>
     </row>
     <row r="46">
@@ -1578,23 +1918,31 @@
           <t>G</t>
         </is>
       </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>Aegypten - Neuseeland</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>26.06.2026</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Aegypten - Iran</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
         <is>
           <t>Aegypten</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="n">
-        <v>0.7</v>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="n">
+        <v>0.48</v>
       </c>
     </row>
     <row r="47">
@@ -1603,22 +1951,30 @@
           <t>H</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>15.06.2026</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>Spanien - Kap Verde</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="E47" s="8" t="n">
+      <c r="G47" s="8" t="n">
         <v>0.85</v>
       </c>
     </row>
@@ -1628,22 +1984,30 @@
           <t>H</t>
         </is>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>15.06.2026</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
         <is>
           <t>Saudi-Arabien - Uruguay</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="E48" s="7" t="inlineStr">
         <is>
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="E48" s="8" t="n">
+      <c r="G48" s="8" t="n">
         <v>0.65</v>
       </c>
     </row>
@@ -1653,22 +2017,30 @@
           <t>H</t>
         </is>
       </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
         <is>
           <t>Spanien - Saudi-Arabien</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
+      <c r="E49" s="7" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="E49" s="8" t="n">
+      <c r="G49" s="8" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -1678,23 +2050,31 @@
           <t>H</t>
         </is>
       </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>Spanien - Uruguay</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>Spanien</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="n">
-        <v>0.6</v>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>21.06.2026</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Kap Verde - Uruguay</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="n">
+        <v>0.72</v>
       </c>
     </row>
     <row r="51">
@@ -1703,23 +2083,31 @@
           <t>H</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Kap Verde - Saudi-Arabien</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>Saudi-Arabien</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>0:1</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="n">
-        <v>0.45</v>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>26.06.2026</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Spanien - Uruguay</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="52">
@@ -1728,23 +2116,31 @@
           <t>H</t>
         </is>
       </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>Kap Verde - Uruguay</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>Uruguay</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>0:2</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="n">
-        <v>0.72</v>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>26.06.2026</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Kap Verde - Saudi-Arabien</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Saudi-Arabien</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="53">
@@ -1753,22 +2149,30 @@
           <t>I</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>16.06.2026</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
         <is>
           <t>Frankreich - Senegal</t>
         </is>
       </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="E53" s="7" t="inlineStr">
         <is>
           <t>Frankreich</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E53" s="8" t="n">
+      <c r="G53" s="8" t="n">
         <v>0.58</v>
       </c>
     </row>
@@ -1778,22 +2182,30 @@
           <t>I</t>
         </is>
       </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>16.06.2026</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>Irak - Norwegen</t>
         </is>
       </c>
-      <c r="C54" s="7" t="inlineStr">
+      <c r="E54" s="7" t="inlineStr">
         <is>
           <t>Norwegen</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="E54" s="8" t="n">
+      <c r="G54" s="8" t="n">
         <v>0.68</v>
       </c>
     </row>
@@ -1803,22 +2215,30 @@
           <t>I</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>22.06.2026</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
         <is>
           <t>Frankreich - Irak</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="E55" s="7" t="inlineStr">
         <is>
           <t>Frankreich</t>
         </is>
       </c>
-      <c r="D55" s="6" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="E55" s="8" t="n">
+      <c r="G55" s="8" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -1828,23 +2248,31 @@
           <t>I</t>
         </is>
       </c>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>Frankreich - Norwegen</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>Frankreich</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="n">
-        <v>0.55</v>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>22.06.2026</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Senegal - Norwegen</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Norwegen</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="G56" s="8" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="57">
@@ -1853,23 +2281,31 @@
           <t>I</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>Senegal - Irak</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
-        <is>
-          <t>Senegal</t>
-        </is>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="n">
-        <v>0.7</v>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>26.06.2026</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Frankreich - Norwegen</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Frankreich</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="G57" s="8" t="n">
+        <v>0.55</v>
       </c>
     </row>
     <row r="58">
@@ -1878,23 +2314,31 @@
           <t>I</t>
         </is>
       </c>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>Senegal - Norwegen</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="inlineStr">
-        <is>
-          <t>Norwegen</t>
-        </is>
-      </c>
-      <c r="D58" s="6" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="n">
-        <v>0.5</v>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>26.06.2026</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Senegal - Irak</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="G58" s="8" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="59">
@@ -1903,22 +2347,30 @@
           <t>J</t>
         </is>
       </c>
-      <c r="B59" s="7" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>16.06.2026</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
         <is>
           <t>Argentinien - Algerien</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
+      <c r="E59" s="7" t="inlineStr">
         <is>
           <t>Argentinien</t>
         </is>
       </c>
-      <c r="D59" s="6" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E59" s="8" t="n">
+      <c r="G59" s="8" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -1928,22 +2380,30 @@
           <t>J</t>
         </is>
       </c>
-      <c r="B60" s="7" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>16.06.2026</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
         <is>
           <t>Oesterreich - Jordanien</t>
         </is>
       </c>
-      <c r="C60" s="7" t="inlineStr">
+      <c r="E60" s="7" t="inlineStr">
         <is>
           <t>Oesterreich</t>
         </is>
       </c>
-      <c r="D60" s="6" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E60" s="8" t="n">
+      <c r="G60" s="8" t="n">
         <v>0.68</v>
       </c>
     </row>
@@ -1953,22 +2413,30 @@
           <t>J</t>
         </is>
       </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>22.06.2026</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
         <is>
           <t>Argentinien - Oesterreich</t>
         </is>
       </c>
-      <c r="C61" s="7" t="inlineStr">
+      <c r="E61" s="7" t="inlineStr">
         <is>
           <t>Argentinien</t>
         </is>
       </c>
-      <c r="D61" s="6" t="inlineStr">
+      <c r="F61" s="6" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E61" s="8" t="n">
+      <c r="G61" s="8" t="n">
         <v>0.65</v>
       </c>
     </row>
@@ -1978,23 +2446,31 @@
           <t>J</t>
         </is>
       </c>
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>Argentinien - Jordanien</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="inlineStr">
-        <is>
-          <t>Argentinien</t>
-        </is>
-      </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>3:0</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="n">
-        <v>0.85</v>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>22.06.2026</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>Algerien - Jordanien</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Algerien</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="G62" s="8" t="n">
+        <v>0.65</v>
       </c>
     </row>
     <row r="63">
@@ -2003,23 +2479,31 @@
           <t>J</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
-        <is>
-          <t>Algerien - Oesterreich</t>
-        </is>
-      </c>
-      <c r="C63" s="7" t="inlineStr">
-        <is>
-          <t>Oesterreich</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="n">
-        <v>0.5</v>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>27.06.2026</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Argentinien - Jordanien</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Argentinien</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="G63" s="8" t="n">
+        <v>0.85</v>
       </c>
     </row>
     <row r="64">
@@ -2028,23 +2512,31 @@
           <t>J</t>
         </is>
       </c>
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>Algerien - Jordanien</t>
-        </is>
-      </c>
-      <c r="C64" s="7" t="inlineStr">
-        <is>
-          <t>Algerien</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="n">
-        <v>0.65</v>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>27.06.2026</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Algerien - Oesterreich</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Oesterreich</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="G64" s="8" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="65">
@@ -2053,22 +2545,30 @@
           <t>K</t>
         </is>
       </c>
-      <c r="B65" s="7" t="inlineStr">
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>17.06.2026</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
         <is>
           <t>Portugal - DR Kongo</t>
         </is>
       </c>
-      <c r="C65" s="7" t="inlineStr">
+      <c r="E65" s="7" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
+      <c r="F65" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E65" s="8" t="n">
+      <c r="G65" s="8" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -2078,22 +2578,30 @@
           <t>K</t>
         </is>
       </c>
-      <c r="B66" s="7" t="inlineStr">
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>17.06.2026</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
         <is>
           <t>Usbekistan - Kolumbien</t>
         </is>
       </c>
-      <c r="C66" s="7" t="inlineStr">
+      <c r="E66" s="7" t="inlineStr">
         <is>
           <t>Kolumbien</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
+      <c r="F66" s="6" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="E66" s="8" t="n">
+      <c r="G66" s="8" t="n">
         <v>0.65</v>
       </c>
     </row>
@@ -2103,22 +2611,30 @@
           <t>K</t>
         </is>
       </c>
-      <c r="B67" s="7" t="inlineStr">
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>23.06.2026</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
         <is>
           <t>Portugal - Usbekistan</t>
         </is>
       </c>
-      <c r="C67" s="7" t="inlineStr">
+      <c r="E67" s="7" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="D67" s="6" t="inlineStr">
+      <c r="F67" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E67" s="8" t="n">
+      <c r="G67" s="8" t="n">
         <v>0.72</v>
       </c>
     </row>
@@ -2128,23 +2644,31 @@
           <t>K</t>
         </is>
       </c>
-      <c r="B68" s="7" t="inlineStr">
-        <is>
-          <t>Portugal - Kolumbien</t>
-        </is>
-      </c>
-      <c r="C68" s="7" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="D68" s="6" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="n">
-        <v>0.52</v>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>23.06.2026</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>DR Kongo - Kolumbien</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Kolumbien</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="G68" s="8" t="n">
+        <v>0.68</v>
       </c>
     </row>
     <row r="69">
@@ -2153,22 +2677,30 @@
           <t>K</t>
         </is>
       </c>
-      <c r="B69" s="7" t="inlineStr">
-        <is>
-          <t>DR Kongo - Usbekistan</t>
-        </is>
-      </c>
-      <c r="C69" s="7" t="inlineStr">
-        <is>
-          <t>DR Kongo</t>
-        </is>
-      </c>
-      <c r="D69" s="6" t="inlineStr">
-        <is>
-          <t>1:0</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="n">
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>27.06.2026</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Portugal - Kolumbien</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="G69" s="8" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -2178,23 +2710,31 @@
           <t>K</t>
         </is>
       </c>
-      <c r="B70" s="7" t="inlineStr">
-        <is>
-          <t>DR Kongo - Kolumbien</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="inlineStr">
-        <is>
-          <t>Kolumbien</t>
-        </is>
-      </c>
-      <c r="D70" s="6" t="inlineStr">
-        <is>
-          <t>0:2</t>
-        </is>
-      </c>
-      <c r="E70" s="8" t="n">
-        <v>0.68</v>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>27.06.2026</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>DR Kongo - Usbekistan</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="G70" s="8" t="n">
+        <v>0.52</v>
       </c>
     </row>
     <row r="71">
@@ -2203,22 +2743,30 @@
           <t>L</t>
         </is>
       </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>17.06.2026</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
         <is>
           <t>England - Kroatien</t>
         </is>
       </c>
-      <c r="C71" s="7" t="inlineStr">
+      <c r="E71" s="7" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="D71" s="6" t="inlineStr">
+      <c r="F71" s="6" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="E71" s="8" t="n">
+      <c r="G71" s="8" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2228,22 +2776,30 @@
           <t>L</t>
         </is>
       </c>
-      <c r="B72" s="7" t="inlineStr">
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>17.06.2026</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
         <is>
           <t>Ghana - Panama</t>
         </is>
       </c>
-      <c r="C72" s="7" t="inlineStr">
+      <c r="E72" s="7" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="D72" s="6" t="inlineStr">
+      <c r="F72" s="6" t="inlineStr">
         <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="E72" s="8" t="n">
+      <c r="G72" s="8" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2253,22 +2809,30 @@
           <t>L</t>
         </is>
       </c>
-      <c r="B73" s="7" t="inlineStr">
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>23.06.2026</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
         <is>
           <t>England - Ghana</t>
         </is>
       </c>
-      <c r="C73" s="7" t="inlineStr">
+      <c r="E73" s="7" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="D73" s="6" t="inlineStr">
+      <c r="F73" s="6" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
-      <c r="E73" s="8" t="n">
+      <c r="G73" s="8" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -2278,23 +2842,31 @@
           <t>L</t>
         </is>
       </c>
-      <c r="B74" s="7" t="inlineStr">
-        <is>
-          <t>England - Panama</t>
-        </is>
-      </c>
-      <c r="C74" s="7" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>3:0</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="n">
-        <v>0.82</v>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>23.06.2026</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>Kroatien - Panama</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>Kroatien</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="G74" s="8" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="75">
@@ -2303,23 +2875,31 @@
           <t>L</t>
         </is>
       </c>
-      <c r="B75" s="7" t="inlineStr">
-        <is>
-          <t>Kroatien - Ghana</t>
-        </is>
-      </c>
-      <c r="C75" s="7" t="inlineStr">
-        <is>
-          <t>Kroatien</t>
-        </is>
-      </c>
-      <c r="D75" s="6" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="n">
-        <v>0.58</v>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>27.06.2026</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>England - Panama</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="G75" s="8" t="n">
+        <v>0.82</v>
       </c>
     </row>
     <row r="76">
@@ -2328,23 +2908,31 @@
           <t>L</t>
         </is>
       </c>
-      <c r="B76" s="7" t="inlineStr">
-        <is>
-          <t>Kroatien - Panama</t>
-        </is>
-      </c>
-      <c r="C76" s="7" t="inlineStr">
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>27.06.2026</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Kroatien - Ghana</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
         <is>
           <t>Kroatien</t>
         </is>
       </c>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="E76" s="8" t="n">
-        <v>0.7</v>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="G76" s="8" t="n">
+        <v>0.58</v>
       </c>
     </row>
   </sheetData>
@@ -2744,12 +3332,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2774,10 +3363,15 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t>Prognose</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Wertigkeit</t>
         </is>
@@ -2786,203 +3380,288 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Halbfinale 1</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Argentinien schlaegt Spanien</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>0.4</v>
+          <t>Achtelfinale (Best 32)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>28.06.-03.07.2026</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Topnationen ziehen ein</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Halbfinale 2</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Frankreich schlaegt England</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>0.38</v>
+          <t>Achtelfinale (Best 16)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>04.07.-07.07.2026</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>ARG, FRA, ESP, ENG, BRA, POR, GER, NED</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Spiel um Platz 3</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Spanien - England 2:1</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>0.35</v>
+          <t>Viertelfinale</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>09.07.-11.07.2026</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ARG, FRA, ESP, ENG weiter</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Finale</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Argentinien - Frankreich</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>0.33</v>
+          <t>Halbfinale 1</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>14.07.2026</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Argentinien schlaegt Spanien</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
+          <t>Halbfinale 2</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>15.07.2026</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Frankreich schlaegt England</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Spiel um Platz 3</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>18.07.2026</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Spanien - England 2:1</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Finale</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>19.07.2026</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Argentinien - Frankreich</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>Weltmeister 2026</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>19.07.2026</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Argentinien (Finalsieg 2:1)</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="D12" s="8" t="n">
         <v>0.3</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Titel-Favoriten-Ranking</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Rang</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Titelchance</t>
         </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Argentinien</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>0.22</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Frankreich</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Spanien</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="n">
-        <v>0.15</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Argentinien</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>0.12</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Brasilien</t>
+          <t>Frankreich</t>
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Spanien</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>England</t>
         </is>
       </c>
       <c r="C19" s="8" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Brasilien</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C23" s="8" t="n">
         <v>0.04</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WM 2026 Prognose: echte Ergebnisse 11./12.06. korrigiert (Kanada-Bosnien 1:1, USA-Paraguay 4:1) und Gruppen A/B/D neu kalibriert
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.55</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="8">
@@ -682,11 +682,11 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="G8" s="8" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="9">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="G10" s="8" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="11">
@@ -776,12 +776,12 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Bosnien-Herz. (gespielt)</t>
+          <t>Unentschieden (gespielt)</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>0:5</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="G13" s="8" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="14">
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="G14" s="8" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="15">
@@ -910,16 +910,16 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Schweiz</t>
+          <t>Unentschieden</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="G15" s="8" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="16">
@@ -1154,36 +1154,38 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>12.06.2026</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C23" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>USA - Paraguay</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="n">
-        <v>0.52</v>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>USA (gespielt)</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1249,7 +1251,7 @@
         </is>
       </c>
       <c r="G25" s="8" t="n">
-        <v>0.62</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="26">
@@ -1282,7 +1284,7 @@
         </is>
       </c>
       <c r="G26" s="8" t="n">
-        <v>0.53</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="27">
@@ -1306,16 +1308,16 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Tuerkei</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="G27" s="8" t="n">
-        <v>0.48</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="28">
@@ -1348,7 +1350,7 @@
         </is>
       </c>
       <c r="G28" s="8" t="n">
-        <v>0.52</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="29">
@@ -3083,12 +3085,12 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
           <t>Tuerkei</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>USA</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Numbers-Variante (.numbers) ergaenzt; gemeinsames Datenmodul wm_data.py als Single Source of Truth
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -505,14 +505,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>WM 2026 – Prognose: noch zu spielende Gruppenspiele</t>
+          <t>WM 2026 – Prognose der Gruppenspiele</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Stand 12.06.2026 · Wertigkeit = subjektive Verlaesslichkeit des Tipps (keine echte Wahrscheinlichkeit)</t>
+          <t>Stand 13. Juni 2026 (nach den Spielen vom 11./12.06.) · Wertigkeit = subjektive Verlässlichkeit des Tipps (keine echte Wahrscheinlichkeit)</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Mexiko - Suedafrika</t>
+          <t>Mexiko - Südafrika</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -604,12 +604,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Suedkorea - Tschechien</t>
+          <t>Südkorea - Tschechien</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Suedkorea (gespielt)</t>
+          <t>Südkorea (gespielt)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Mexiko - Suedkorea</t>
+          <t>Mexiko - Südkorea</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Tschechien - Suedafrika</t>
+          <t>Tschechien - Südafrika</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -738,12 +738,12 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Suedkorea - Suedafrika</t>
+          <t>Südkorea - Südafrika</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Suedkorea</t>
+          <t>Südkorea</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -1204,12 +1204,12 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Australien - Tuerkei</t>
+          <t>Australien - Türkei</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Tuerkei</t>
+          <t>Türkei</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Paraguay - Tuerkei</t>
+          <t>Paraguay - Türkei</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Tuerkei</t>
+          <t>Türkei</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>USA - Tuerkei</t>
+          <t>USA - Türkei</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Deutschland - Curacao</t>
+          <t>Deutschland - Curaçao</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Elfenbeinkueste - Ecuador</t>
+          <t>Elfenbeinküste - Ecuador</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Deutschland - Elfenbeinkueste</t>
+          <t>Deutschland - Elfenbeinküste</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Curacao - Ecuador</t>
+          <t>Curaçao - Ecuador</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -1534,12 +1534,12 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Curacao - Elfenbeinkueste</t>
+          <t>Curaçao - Elfenbeinküste</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Elfenbeinkueste</t>
+          <t>Elfenbeinküste</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Belgien - Aegypten</t>
+          <t>Belgien - Ägypten</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -1864,12 +1864,12 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Aegypten - Neuseeland</t>
+          <t>Ägypten - Neuseeland</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>Aegypten</t>
+          <t>Ägypten</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Aegypten - Iran</t>
+          <t>Ägypten - Iran</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>Aegypten</t>
+          <t>Ägypten</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -2392,12 +2392,12 @@
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Oesterreich - Jordanien</t>
+          <t>Österreich - Jordanien</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>Oesterreich</t>
+          <t>Österreich</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Argentinien - Oesterreich</t>
+          <t>Argentinien - Österreich</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
@@ -2524,12 +2524,12 @@
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Algerien - Oesterreich</t>
+          <t>Algerien - Österreich</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Oesterreich</t>
+          <t>Österreich</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
@@ -2939,8 +2939,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3009,7 +3009,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Suedkorea</t>
+          <t>Südkorea</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -3019,7 +3019,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Suedafrika</t>
+          <t>Südafrika</t>
         </is>
       </c>
     </row>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Tuerkei</t>
+          <t>Türkei</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -3122,12 +3122,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Elfenbeinkueste</t>
+          <t>Elfenbeinküste</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Curacao</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Aegypten</t>
+          <t>Ägypten</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Oesterreich</t>
+          <t>Österreich</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -3353,7 +3353,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Exakte Paarungen haengen von Endtabellen + FIFA-Zuordnung der 8 besten Dritten ab und sind nicht serioes vorab fixierbar.</t>
+          <t>Exakte Paarungen hängen von Endtabellen + FIFA-Zuordnung der 8 besten Dritten ab und sind nicht seriös vorab fixierbar.</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>28.06.-03.07.2026</t>
+          <t>28.06.–03.07.2026</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>04.07.-07.07.2026</t>
+          <t>04.07.–07.07.2026</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>09.07.-11.07.2026</t>
+          <t>09.07.–11.07.2026</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Argentinien schlaegt Spanien</t>
+          <t>Argentinien schlägt Spanien</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Frankreich schlaegt England</t>
+          <t>Frankreich schlägt England</t>
         </is>
       </c>
       <c r="D9" s="8" t="n">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Spanien - England 2:1</t>
+          <t>Spanien – England 2:1</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Argentinien - Frankreich</t>
+          <t>Argentinien – Frankreich</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
@@ -3669,8 +3669,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel: AutoFilter (Sortieren/Filtern) in Kopfzeile von Gruppenphase und Gruppentabellen
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -11,7 +11,10 @@
     <sheet name="Gruppentabellen-Prognose" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="K.-o.-Prognose" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gruppenphase'!$A$4:$G$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Gruppentabellen-Prognose'!$A$3:$E$15</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -2938,6 +2941,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:G76"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
@@ -3321,6 +3325,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:E15"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Prognosen quoten-/ranking-kalibriert (Buchmacher 06/2026 + FIFA-Rangliste); Markdown jetzt ebenfalls generiert (build_md.py)
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Stand 13. Juni 2026 (nach den Spielen vom 11./12.06.) · Wertigkeit = subjektive Verlässlichkeit des Tipps (keine echte Wahrscheinlichkeit)</t>
+          <t>Stand 13. Juni 2026 (quoten-/ranking-kalibriert, nach den Spielen vom 11./12.06.) · Wertigkeit = subjektive Verlässlichkeit des Tipps (keine echte Wahrscheinlichkeit)</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="G8" s="8" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="9">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="G9" s="8" t="n">
-        <v>0.6</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="10">
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="G10" s="8" t="n">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="11">
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="G12" s="8" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="13">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="G13" s="8" t="n">
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="14">
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="G14" s="8" t="n">
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="15">
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="G16" s="8" t="n">
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="17">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="G19" s="8" t="n">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="20">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="G20" s="8" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="21">
@@ -1120,7 +1120,7 @@
         </is>
       </c>
       <c r="G21" s="8" t="n">
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="22">
@@ -1153,7 +1153,7 @@
         </is>
       </c>
       <c r="G22" s="8" t="n">
-        <v>0.75</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="23">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="G25" s="8" t="n">
-        <v>0.65</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="26">
@@ -1320,7 +1320,7 @@
         </is>
       </c>
       <c r="G27" s="8" t="n">
-        <v>0.52</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="28">
@@ -1386,7 +1386,7 @@
         </is>
       </c>
       <c r="G29" s="8" t="n">
-        <v>0.85</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="30">
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="G33" s="8" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="34">
@@ -1551,7 +1551,7 @@
         </is>
       </c>
       <c r="G34" s="8" t="n">
-        <v>0.75</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="35">
@@ -1584,7 +1584,7 @@
         </is>
       </c>
       <c r="G35" s="8" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="36">
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="G37" s="8" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="38">
@@ -1683,7 +1683,7 @@
         </is>
       </c>
       <c r="G38" s="8" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="39">
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="G39" s="8" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="40">
@@ -1782,7 +1782,7 @@
         </is>
       </c>
       <c r="G41" s="8" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="42">
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="G42" s="8" t="n">
-        <v>0.68</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="43">
@@ -1848,7 +1848,7 @@
         </is>
       </c>
       <c r="G43" s="8" t="n">
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="44">
@@ -1914,7 +1914,7 @@
         </is>
       </c>
       <c r="G45" s="8" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="46">
@@ -1980,7 +1980,7 @@
         </is>
       </c>
       <c r="G47" s="8" t="n">
-        <v>0.85</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="48">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="G48" s="8" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="49">
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="G49" s="8" t="n">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="50">
@@ -2079,7 +2079,7 @@
         </is>
       </c>
       <c r="G50" s="8" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="51">
@@ -2112,7 +2112,7 @@
         </is>
       </c>
       <c r="G51" s="8" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="52">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="G52" s="8" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="53">
@@ -2211,7 +2211,7 @@
         </is>
       </c>
       <c r="G54" s="8" t="n">
-        <v>0.68</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="55">
@@ -2244,7 +2244,7 @@
         </is>
       </c>
       <c r="G55" s="8" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="56">
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="G57" s="8" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="58">
@@ -2343,7 +2343,7 @@
         </is>
       </c>
       <c r="G58" s="8" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="59">
@@ -2376,7 +2376,7 @@
         </is>
       </c>
       <c r="G59" s="8" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="60">
@@ -2442,7 +2442,7 @@
         </is>
       </c>
       <c r="G61" s="8" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="62">
@@ -2475,7 +2475,7 @@
         </is>
       </c>
       <c r="G62" s="8" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="63">
@@ -2508,7 +2508,7 @@
         </is>
       </c>
       <c r="G63" s="8" t="n">
-        <v>0.85</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="64">
@@ -2574,7 +2574,7 @@
         </is>
       </c>
       <c r="G65" s="8" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="66">
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="G66" s="8" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="67">
@@ -2640,7 +2640,7 @@
         </is>
       </c>
       <c r="G67" s="8" t="n">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="68">
@@ -2706,7 +2706,7 @@
         </is>
       </c>
       <c r="G69" s="8" t="n">
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="70">
@@ -2772,7 +2772,7 @@
         </is>
       </c>
       <c r="G71" s="8" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="72">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="G72" s="8" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="73">
@@ -2838,7 +2838,7 @@
         </is>
       </c>
       <c r="G73" s="8" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="74">
@@ -2871,7 +2871,7 @@
         </is>
       </c>
       <c r="G74" s="8" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="75">
@@ -2904,7 +2904,7 @@
         </is>
       </c>
       <c r="G75" s="8" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="76">
@@ -3401,7 +3401,7 @@
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="6">
@@ -3417,11 +3417,11 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>ARG, FRA, ESP, ENG, BRA, POR, GER, NED</t>
+          <t>ESP, FRA, ENG, BRA, ARG, GER, POR, NED</t>
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="7">
@@ -3437,11 +3437,11 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ARG, FRA, ESP, ENG weiter</t>
+          <t>Spanien, Frankreich, England, Argentinien</t>
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="8">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Argentinien schlägt Spanien</t>
+          <t>Spanien schlägt Argentinien</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
@@ -3481,7 +3481,7 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="10">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Spanien – England 2:1</t>
+          <t>Argentinien – England 2:1</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
@@ -3517,11 +3517,11 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Argentinien – Frankreich</t>
+          <t>Spanien – Frankreich</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="12">
@@ -3537,11 +3537,11 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Argentinien (Finalsieg 2:1)</t>
+          <t>Spanien (Finalsieg 2:1)</t>
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="14">
@@ -3574,11 +3574,11 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Argentinien</t>
+          <t>Spanien</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>0.22</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="17">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="18">
@@ -3600,11 +3600,11 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Spanien</t>
+          <t>England</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>0.15</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="19">
@@ -3613,11 +3613,11 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Brasilien</t>
         </is>
       </c>
       <c r="C19" s="8" t="n">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="20">
@@ -3626,11 +3626,11 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Brasilien</t>
+          <t>Argentinien</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="21">
@@ -3639,11 +3639,11 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="C21" s="8" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="22">
@@ -3652,11 +3652,11 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
Halbzeit-Prognose (HZ-Fuehrung/Ergebnis/Wertigkeit) ergaenzt; sync-jetzt.command als Ein-Klick-Sync-Button
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -12,7 +12,7 @@
     <sheet name="K.-o.-Prognose" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gruppenphase'!$A$4:$G$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gruppenphase'!$A$4:$J$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Gruppentabellen-Prognose'!$A$3:$E$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,10 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -555,6 +558,21 @@
           <t>Wertigkeit</t>
         </is>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>HZ-Führung</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>HZ-Ergebnis</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>HZ-Wert.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -590,6 +608,21 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Mexiko</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -625,6 +658,21 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -658,6 +706,19 @@
       <c r="G7" s="8" t="n">
         <v>0.52</v>
       </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -691,6 +752,19 @@
       <c r="G8" s="8" t="n">
         <v>0.66</v>
       </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Tschechien</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>0.54</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -724,6 +798,19 @@
       <c r="G9" s="8" t="n">
         <v>0.64</v>
       </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Mexiko</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -757,6 +844,19 @@
       <c r="G10" s="8" t="n">
         <v>0.72</v>
       </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Südkorea</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -792,6 +892,21 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Bosnien-Herz.</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -825,6 +940,19 @@
       <c r="G12" s="8" t="n">
         <v>0.72</v>
       </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Schweiz</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -858,6 +986,19 @@
       <c r="G13" s="8" t="n">
         <v>0.64</v>
       </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Kanada</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -891,6 +1032,19 @@
       <c r="G14" s="8" t="n">
         <v>0.54</v>
       </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -924,6 +1078,19 @@
       <c r="G15" s="8" t="n">
         <v>0.45</v>
       </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -957,6 +1124,19 @@
       <c r="G16" s="8" t="n">
         <v>0.64</v>
       </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Bosnien-Herz.</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -990,6 +1170,19 @@
       <c r="G17" s="8" t="n">
         <v>0.55</v>
       </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1023,6 +1216,19 @@
       <c r="G18" s="8" t="n">
         <v>0.62</v>
       </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Schottland</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -1056,6 +1262,19 @@
       <c r="G19" s="8" t="n">
         <v>0.83</v>
       </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Brasilien</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1089,6 +1308,19 @@
       <c r="G20" s="8" t="n">
         <v>0.58</v>
       </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -1122,6 +1354,19 @@
       <c r="G21" s="8" t="n">
         <v>0.74</v>
       </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Brasilien</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="n">
+        <v>0.62</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -1155,6 +1400,19 @@
       <c r="G22" s="8" t="n">
         <v>0.77</v>
       </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>0.65</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1190,6 +1448,21 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1223,6 +1496,19 @@
       <c r="G24" s="8" t="n">
         <v>0.55</v>
       </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -1256,6 +1542,19 @@
       <c r="G25" s="8" t="n">
         <v>0.7</v>
       </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="n">
+        <v>0.58</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -1289,6 +1588,19 @@
       <c r="G26" s="8" t="n">
         <v>0.55</v>
       </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -1322,6 +1634,19 @@
       <c r="G27" s="8" t="n">
         <v>0.55</v>
       </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J27" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -1355,6 +1680,19 @@
       <c r="G28" s="8" t="n">
         <v>0.5</v>
       </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J28" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -1388,6 +1726,19 @@
       <c r="G29" s="8" t="n">
         <v>0.88</v>
       </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J29" s="8" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -1421,6 +1772,19 @@
       <c r="G30" s="8" t="n">
         <v>0.5</v>
       </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J30" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -1454,6 +1818,19 @@
       <c r="G31" s="8" t="n">
         <v>0.62</v>
       </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J31" s="8" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -1487,6 +1864,19 @@
       <c r="G32" s="8" t="n">
         <v>0.78</v>
       </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="J32" s="8" t="n">
+        <v>0.66</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -1520,6 +1910,19 @@
       <c r="G33" s="8" t="n">
         <v>0.6</v>
       </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J33" s="8" t="n">
+        <v>0.48</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -1553,6 +1956,19 @@
       <c r="G34" s="8" t="n">
         <v>0.77</v>
       </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Elfenbeinküste</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="n">
+        <v>0.65</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -1586,6 +2002,19 @@
       <c r="G35" s="8" t="n">
         <v>0.6</v>
       </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Niederlande</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J35" s="8" t="n">
+        <v>0.48</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -1619,6 +2048,19 @@
       <c r="G36" s="8" t="n">
         <v>0.55</v>
       </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J36" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -1652,6 +2094,19 @@
       <c r="G37" s="8" t="n">
         <v>0.62</v>
       </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Niederlande</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J37" s="8" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -1685,6 +2140,19 @@
       <c r="G38" s="8" t="n">
         <v>0.66</v>
       </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J38" s="8" t="n">
+        <v>0.54</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -1718,6 +2186,19 @@
       <c r="G39" s="8" t="n">
         <v>0.74</v>
       </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Niederlande</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J39" s="8" t="n">
+        <v>0.62</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -1751,6 +2232,19 @@
       <c r="G40" s="8" t="n">
         <v>0.52</v>
       </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J40" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -1784,6 +2278,19 @@
       <c r="G41" s="8" t="n">
         <v>0.62</v>
       </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J41" s="8" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -1817,6 +2324,19 @@
       <c r="G42" s="8" t="n">
         <v>0.7</v>
       </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J42" s="8" t="n">
+        <v>0.58</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -1850,6 +2370,19 @@
       <c r="G43" s="8" t="n">
         <v>0.64</v>
       </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J43" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -1883,6 +2416,19 @@
       <c r="G44" s="8" t="n">
         <v>0.7</v>
       </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Ägypten</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J44" s="8" t="n">
+        <v>0.58</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -1916,6 +2462,19 @@
       <c r="G45" s="8" t="n">
         <v>0.85</v>
       </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J45" s="8" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -1949,6 +2508,19 @@
       <c r="G46" s="8" t="n">
         <v>0.48</v>
       </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J46" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -1982,6 +2554,19 @@
       <c r="G47" s="8" t="n">
         <v>0.88</v>
       </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J47" s="8" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -2015,6 +2600,19 @@
       <c r="G48" s="8" t="n">
         <v>0.66</v>
       </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="J48" s="8" t="n">
+        <v>0.54</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -2048,6 +2646,19 @@
       <c r="G49" s="8" t="n">
         <v>0.83</v>
       </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J49" s="8" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
@@ -2081,6 +2692,19 @@
       <c r="G50" s="8" t="n">
         <v>0.73</v>
       </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="J50" s="8" t="n">
+        <v>0.61</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -2114,6 +2738,19 @@
       <c r="G51" s="8" t="n">
         <v>0.62</v>
       </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J51" s="8" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -2147,6 +2784,19 @@
       <c r="G52" s="8" t="n">
         <v>0.46</v>
       </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J52" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -2180,6 +2830,19 @@
       <c r="G53" s="8" t="n">
         <v>0.58</v>
       </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J53" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
@@ -2213,6 +2876,19 @@
       <c r="G54" s="8" t="n">
         <v>0.7</v>
       </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>Norwegen</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="J54" s="8" t="n">
+        <v>0.58</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -2246,6 +2922,19 @@
       <c r="G55" s="8" t="n">
         <v>0.82</v>
       </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>Frankreich</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J55" s="8" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -2279,6 +2968,19 @@
       <c r="G56" s="8" t="n">
         <v>0.5</v>
       </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J56" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -2312,6 +3014,19 @@
       <c r="G57" s="8" t="n">
         <v>0.5600000000000001</v>
       </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J57" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -2345,6 +3060,19 @@
       <c r="G58" s="8" t="n">
         <v>0.72</v>
       </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J58" s="8" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
@@ -2378,6 +3106,19 @@
       <c r="G59" s="8" t="n">
         <v>0.72</v>
       </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>Argentinien</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J59" s="8" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -2411,6 +3152,19 @@
       <c r="G60" s="8" t="n">
         <v>0.68</v>
       </c>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>Österreich</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J60" s="8" t="n">
+        <v>0.5600000000000001</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
@@ -2444,6 +3198,19 @@
       <c r="G61" s="8" t="n">
         <v>0.66</v>
       </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>Argentinien</t>
+        </is>
+      </c>
+      <c r="I61" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J61" s="8" t="n">
+        <v>0.54</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
@@ -2477,6 +3244,19 @@
       <c r="G62" s="8" t="n">
         <v>0.64</v>
       </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>Algerien</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J62" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
@@ -2510,6 +3290,19 @@
       <c r="G63" s="8" t="n">
         <v>0.88</v>
       </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>Argentinien</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J63" s="8" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
@@ -2543,6 +3336,19 @@
       <c r="G64" s="8" t="n">
         <v>0.5</v>
       </c>
+      <c r="H64" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J64" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -2576,6 +3382,19 @@
       <c r="G65" s="8" t="n">
         <v>0.72</v>
       </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J65" s="8" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
@@ -2609,6 +3428,19 @@
       <c r="G66" s="8" t="n">
         <v>0.66</v>
       </c>
+      <c r="H66" s="7" t="inlineStr">
+        <is>
+          <t>Kolumbien</t>
+        </is>
+      </c>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="J66" s="8" t="n">
+        <v>0.54</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
@@ -2642,6 +3474,19 @@
       <c r="G67" s="8" t="n">
         <v>0.75</v>
       </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J67" s="8" t="n">
+        <v>0.63</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -2675,6 +3520,19 @@
       <c r="G68" s="8" t="n">
         <v>0.68</v>
       </c>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>Kolumbien</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="J68" s="8" t="n">
+        <v>0.5600000000000001</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -2708,6 +3566,19 @@
       <c r="G69" s="8" t="n">
         <v>0.54</v>
       </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J69" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
@@ -2741,6 +3612,19 @@
       <c r="G70" s="8" t="n">
         <v>0.52</v>
       </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J70" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
@@ -2774,6 +3658,19 @@
       <c r="G71" s="8" t="n">
         <v>0.5600000000000001</v>
       </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J71" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -2807,6 +3704,19 @@
       <c r="G72" s="8" t="n">
         <v>0.5600000000000001</v>
       </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J72" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
@@ -2840,6 +3750,19 @@
       <c r="G73" s="8" t="n">
         <v>0.72</v>
       </c>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J73" s="8" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
@@ -2873,6 +3796,19 @@
       <c r="G74" s="8" t="n">
         <v>0.72</v>
       </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>Kroatien</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J74" s="8" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -2906,6 +3842,19 @@
       <c r="G75" s="8" t="n">
         <v>0.85</v>
       </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J75" s="8" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
@@ -2939,12 +3888,25 @@
       <c r="G76" s="8" t="n">
         <v>0.58</v>
       </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J76" s="8" t="n">
+        <v>0.52</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G76"/>
+  <autoFilter ref="A4:J76"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Transfermarkt-Kaderwerte einbezogen: Titelrennen aktualisiert (Frankreich knapp vor Spanien)
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -518,7 +518,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Stand 13. Juni 2026 (quoten-/ranking-kalibriert, nach den Spielen vom 11./12.06.) · Wertigkeit = subjektive Verlässlichkeit des Tipps (keine echte Wahrscheinlichkeit)</t>
+          <t>Stand 13. Juni 2026 (kalibriert mit Buchmacher-Quoten, FIFA-Rangliste &amp; Transfermarkt-Kaderwerten; nach den Spielen vom 11./12.06.) · Wertigkeit = subjektive Verlässlichkeit des Tipps (keine echte Wahrscheinlichkeit)</t>
         </is>
       </c>
     </row>
@@ -4379,7 +4379,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>ESP, FRA, ENG, BRA, ARG, GER, POR, NED</t>
+          <t>FRA, ESP, ENG, BRA, ARG, POR, GER, NED</t>
         </is>
       </c>
       <c r="D6" s="8" t="n">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Spanien, Frankreich, England, Argentinien</t>
+          <t>Frankreich, Spanien, England, Argentinien</t>
         </is>
       </c>
       <c r="D7" s="8" t="n">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Spanien – Frankreich</t>
+          <t>Frankreich – Spanien</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Spanien (Finalsieg 2:1)</t>
+          <t>Frankreich (Finalsieg 2:1)</t>
         </is>
       </c>
       <c r="D12" s="8" t="n">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Spanien</t>
+          <t>Frankreich</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Frankreich</t>
+          <t>Spanien</t>
         </is>
       </c>
       <c r="C17" s="8" t="n">
@@ -4566,7 +4566,7 @@
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="19">
@@ -4601,7 +4601,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C21" s="8" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">

</xml_diff>

<commit_message>
Ergebnisse 13.06. eingepflegt (4 Spiele); Gruppe D neu (Australien 2., Tuerkei 3.), HZ-Daten ergaenzt
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -518,7 +518,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Stand 13. Juni 2026 (kalibriert mit Buchmacher-Quoten, FIFA-Rangliste &amp; Transfermarkt-Kaderwerten; nach den Spielen vom 11./12.06.) · Wertigkeit = subjektive Verlässlichkeit des Tipps (keine echte Wahrscheinlichkeit)</t>
+          <t>Stand 14. Juni 2026 (kalibriert mit Buchmacher-Quoten, FIFA-Rangliste &amp; Transfermarkt-Kaderwerten; nach den Spielen vom 11.–13.06.) · Wertigkeit = subjektive Verlässlichkeit des Tipps (keine echte Wahrscheinlichkeit)</t>
         </is>
       </c>
     </row>
@@ -909,49 +909,53 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>13.06.2026</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Katar - Schweiz</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Unentschieden (gespielt)</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Schweiz</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>0:2</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>Schweiz</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>0:1</t>
         </is>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>0.6</v>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1139,95 +1143,103 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>13.06.2026</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Brasilien - Marokko</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Brasilien</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Unentschieden (gespielt)</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>Unentschieden</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>0:0</t>
-        </is>
-      </c>
-      <c r="J17" s="8" t="n">
-        <v>0.52</v>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>13.06.2026</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Haiti - Schottland</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Schottland (gespielt)</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>Schottland</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>0:2</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>Schottland</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>0:1</t>
         </is>
       </c>
-      <c r="J18" s="8" t="n">
-        <v>0.5</v>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -1465,49 +1477,53 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>13.06.2026</t>
         </is>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Australien - Türkei</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Türkei</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="H24" s="7" t="inlineStr">
-        <is>
-          <t>Unentschieden</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>0:0</t>
-        </is>
-      </c>
-      <c r="J24" s="8" t="n">
-        <v>0.52</v>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Australien (gespielt)</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Australien</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1536,24 +1552,24 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="G25" s="8" t="n">
-        <v>0.7</v>
+        <v>0.58</v>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Unentschieden</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>0:0</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>0.58</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="26">
@@ -1586,7 +1602,7 @@
         </is>
       </c>
       <c r="G26" s="8" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
@@ -1632,7 +1648,7 @@
         </is>
       </c>
       <c r="G27" s="8" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
@@ -1669,16 +1685,16 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Australien</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="G28" s="8" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
@@ -4056,17 +4072,17 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
+          <t>Australien</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
           <t>Türkei</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Australien</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Live-Neuberechnung Deutschland-Curacao aus HZ-Stand 1:1 -> Tipp 3:1 (70%); LIVE_HT-Mechanik ergaenzt
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -1736,24 +1736,26 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="G29" s="8" t="n">
-        <v>0.88</v>
+        <v>0.7</v>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Unentschieden</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="J29" s="8" t="n">
-        <v>0.7</v>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Live-Korrektur Deutschland-Curacao: HZ 3:1, Endergebnis-Tipp 4:1 (85%)
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -1736,20 +1736,20 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
           <t>3:1</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H29" s="7" t="inlineStr">
-        <is>
-          <t>Unentschieden</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>1:1</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Ergebnisse 14.06. (Deutschland 7:1, NED-JPN 2:2); Bilanz-Blatt mit ehrlicher Trefferquote ergaenzt
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Gruppenphase" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Gruppentabellen-Prognose" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="K.-o.-Prognose" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Bilanz" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gruppenphase'!$A$4:$J$76</definedName>
@@ -24,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0 %"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +52,11 @@
       <b val="1"/>
       <color rgb="001F4E78"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -102,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,6 +134,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1711,48 +1718,50 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>14.06.2026</t>
         </is>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C29" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>Deutschland - Curaçao</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Deutschland (gespielt)</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>7:1</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="H29" s="7" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>3:1</t>
         </is>
       </c>
-      <c r="J29" s="6" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1989,49 +1998,53 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>14.06.2026</t>
         </is>
       </c>
-      <c r="C35" s="6" t="n">
+      <c r="C35" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>Niederlande - Japan</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>Niederlande</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="G35" s="8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>Niederlande</t>
-        </is>
-      </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>1:0</t>
-        </is>
-      </c>
-      <c r="J35" s="8" t="n">
-        <v>0.48</v>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Unentschieden (gespielt)</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Unentschieden</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -4659,4 +4672,396 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bilanz – meine bisherige Trefferquote (ehrlich)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Sieger korrekt: 5/9 (~56 %) · Halbzeit-Führung korrekt: 7/9 (~78 %) · Exaktes Ergebnis: 2/9 (~22 %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Begegnung</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Mein Vorab-Tipp</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Echt</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Sieger</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>HZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>11.06.</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Mexiko – Südafrika</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Mexiko 2:0</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>11.06.</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Südkorea – Tschechien</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Südkorea 2:1</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>12.06.</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Kanada – Bosnien-Herz.</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>(Datenfehler)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>12.06.</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>USA – Paraguay</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>USA 2:1</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>13.06.</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Katar – Schweiz</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Schweiz 0:2</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>13.06.</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Brasilien – Marokko</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Brasilien 2:1</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>13.06.</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Haiti – Schottland</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Schottland 0:2</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>13.06.</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Australien – Türkei</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Türkei 2:1</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>0:2 (Australien)</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>14.06.</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Deutschland – Curaçao</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Deutschland 3:0</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>7:1</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>14.06.</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Niederlande – Japan</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Niederlande 2:1</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Alle Ergebnisse bis 14.06. eingepflegt (CIV 1:0 Ecuador, Schweden 5:1); Gruppen E/F neu kalibriert; Bilanz aktualisiert
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -525,7 +525,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Stand 14. Juni 2026 (kalibriert mit Buchmacher-Quoten, FIFA-Rangliste &amp; Transfermarkt-Kaderwerten; nach den Spielen vom 11.–13.06.) · Wertigkeit = subjektive Verlässlichkeit des Tipps (keine echte Wahrscheinlichkeit)</t>
+          <t>Stand 15. Juni 2026 (kalibriert mit Buchmacher-Quoten, FIFA-Rangliste &amp; Transfermarkt-Kaderwerten; nach allen Spielen bis 14.06.) · Wertigkeit = subjektive Verlässlichkeit des Tipps (keine echte Wahrscheinlichkeit)</t>
         </is>
       </c>
     </row>
@@ -1768,49 +1768,53 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>14.06.2026</t>
         </is>
       </c>
-      <c r="C30" s="6" t="n">
+      <c r="C30" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>Elfenbeinküste - Ecuador</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>0:1</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Elfenbeinküste (gespielt)</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>Unentschieden</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>0:0</t>
         </is>
       </c>
-      <c r="J30" s="8" t="n">
-        <v>0.52</v>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1843,20 +1847,20 @@
         </is>
       </c>
       <c r="G31" s="8" t="n">
-        <v>0.62</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Unentschieden</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>0:0</t>
         </is>
       </c>
       <c r="J31" s="8" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="32">
@@ -2048,49 +2052,53 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>14.06.2026</t>
         </is>
       </c>
-      <c r="C36" s="6" t="n">
+      <c r="C36" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>Schweden - Tunesien</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Schweden (gespielt)</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>5:1</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>Schweden</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>1:0</t>
-        </is>
-      </c>
-      <c r="G36" s="8" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="H36" s="7" t="inlineStr">
-        <is>
-          <t>Unentschieden</t>
-        </is>
-      </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>0:0</t>
-        </is>
-      </c>
-      <c r="J36" s="8" t="n">
-        <v>0.52</v>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -2123,20 +2131,20 @@
         </is>
       </c>
       <c r="G37" s="8" t="n">
-        <v>0.62</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>Niederlande</t>
+          <t>Unentschieden</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>0:0</t>
         </is>
       </c>
       <c r="J37" s="8" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="38">
@@ -4114,12 +4122,12 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
+          <t>Elfenbeinküste</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
           <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Elfenbeinküste</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -4141,12 +4149,12 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
+          <t>Schweden</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
           <t>Japan</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Schweden</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -4680,7 +4688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4701,7 +4709,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Sieger korrekt: 5/9 (~56 %) · Halbzeit-Führung korrekt: 7/9 (~78 %) · Exaktes Ergebnis: 2/9 (~22 %)</t>
+          <t>Sieger korrekt: 6/11 (~55 %) · Halbzeit-Führung korrekt: 8/11 (~73 %) · Exaktes Ergebnis: 2/11 (~18 %)</t>
         </is>
       </c>
     </row>
@@ -5033,25 +5041,89 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
+          <t>Elfenbeinküste – Ecuador</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Ecuador 0:1</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>1:0 (Elfenbeinküste)</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>14.06.</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
           <t>Niederlande – Japan</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Niederlande 2:1</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>14.06.</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Schweden – Tunesien</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Schweden 1:0</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>5:1</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>✗</t>
         </is>

</xml_diff>

<commit_message>
Excel: AutoFilter auf allen Blättern (Gruppenphase, Gruppentabellen, Bilanz)
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -14,6 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gruppenphase'!$A$4:$J$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Gruppentabellen-Prognose'!$A$3:$E$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Bilanz'!$A$4:$F$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4442,6 +4444,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:E15"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -5237,6 +5240,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:F16"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Alle Ergebnisse bis 16.06. eingepflegt (8 neue Spiele); Bilanz aktualisiert (Sieger 10/19)
</commit_message>
<xml_diff>
--- a/WM-2026-Prognose.xlsx
+++ b/WM-2026-Prognose.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gruppenphase'!$A$4:$J$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Gruppentabellen-Prognose'!$A$3:$E$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Bilanz'!$A$4:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Bilanz'!$A$4:$F$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -545,7 +545,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Stand 15. Juni 2026 (kalibriert mit Buchmacher-Quoten, FIFA-Rangliste &amp; Transfermarkt-Kaderwerten; nach allen Spielen bis 14.06.) · Fokus: Sieger- &amp; Halbzeit-Tipp + Wertigkeit (Tendenz). Exaktes Ergebnis nur als Nebenangabe.</t>
+          <t>Stand 16. Juni 2026 (kalibriert mit Buchmacher-Quoten, FIFA-Rangliste &amp; Transfermarkt-Kaderwerten; nach allen Spielen bis 16.06.) · Fokus: Sieger- &amp; Halbzeit-Tipp + Wertigkeit (Tendenz). Exaktes Ergebnis nur als Nebenangabe.</t>
         </is>
       </c>
     </row>
@@ -2332,96 +2332,96 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>15.06.2026</t>
         </is>
       </c>
-      <c r="C41" s="8" t="n">
+      <c r="C41" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>Belgien - Ägypten</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>Belgien</t>
         </is>
       </c>
-      <c r="F41" s="9" t="inlineStr">
+      <c r="F41" s="5" t="inlineStr">
         <is>
           <t>Belgien (1:0)</t>
         </is>
       </c>
-      <c r="G41" s="10" t="n">
+      <c r="G41" s="6" t="n">
         <v>0.62</v>
       </c>
-      <c r="H41" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="I41" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="J41" s="8" t="inlineStr">
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="I41" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>15.06.2026</t>
         </is>
       </c>
-      <c r="C42" s="8" t="n">
+      <c r="C42" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D42" s="9" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>Iran - Neuseeland</t>
         </is>
       </c>
-      <c r="E42" s="9" t="inlineStr">
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>Iran</t>
         </is>
       </c>
-      <c r="F42" s="9" t="inlineStr">
+      <c r="F42" s="5" t="inlineStr">
         <is>
           <t>Iran (1:0)</t>
         </is>
       </c>
-      <c r="G42" s="10" t="n">
+      <c r="G42" s="6" t="n">
         <v>0.7</v>
       </c>
-      <c r="H42" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="I42" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="J42" s="8" t="inlineStr">
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
@@ -2620,96 +2620,96 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>15.06.2026</t>
         </is>
       </c>
-      <c r="C47" s="8" t="n">
+      <c r="C47" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>Spanien - Kap Verde</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="F47" s="9" t="inlineStr">
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t>Spanien (2:0)</t>
         </is>
       </c>
-      <c r="G47" s="10" t="n">
+      <c r="G47" s="6" t="n">
         <v>0.88</v>
       </c>
-      <c r="H47" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="I47" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="J47" s="8" t="inlineStr">
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="I47" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>15.06.2026</t>
         </is>
       </c>
-      <c r="C48" s="8" t="n">
+      <c r="C48" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D48" s="9" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>Saudi-Arabien - Uruguay</t>
         </is>
       </c>
-      <c r="E48" s="9" t="inlineStr">
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="F48" s="9" t="inlineStr">
+      <c r="F48" s="5" t="inlineStr">
         <is>
           <t>Uruguay (0:1)</t>
         </is>
       </c>
-      <c r="G48" s="10" t="n">
+      <c r="G48" s="6" t="n">
         <v>0.66</v>
       </c>
-      <c r="H48" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="I48" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="J48" s="8" t="inlineStr">
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
@@ -2908,96 +2908,96 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>16.06.2026</t>
         </is>
       </c>
-      <c r="C53" s="8" t="n">
+      <c r="C53" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D53" s="9" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>Frankreich - Senegal</t>
         </is>
       </c>
-      <c r="E53" s="9" t="inlineStr">
+      <c r="E53" s="5" t="inlineStr">
         <is>
           <t>Frankreich</t>
         </is>
       </c>
-      <c r="F53" s="9" t="inlineStr">
+      <c r="F53" s="5" t="inlineStr">
         <is>
           <t>Unentschieden (0:0)</t>
         </is>
       </c>
-      <c r="G53" s="10" t="n">
+      <c r="G53" s="6" t="n">
         <v>0.58</v>
       </c>
-      <c r="H53" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="I53" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="J53" s="8" t="inlineStr">
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>16.06.2026</t>
         </is>
       </c>
-      <c r="C54" s="8" t="n">
+      <c r="C54" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D54" s="9" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>Irak - Norwegen</t>
         </is>
       </c>
-      <c r="E54" s="9" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>Norwegen</t>
         </is>
       </c>
-      <c r="F54" s="9" t="inlineStr">
+      <c r="F54" s="5" t="inlineStr">
         <is>
           <t>Norwegen (0:1)</t>
         </is>
       </c>
-      <c r="G54" s="10" t="n">
+      <c r="G54" s="6" t="n">
         <v>0.7</v>
       </c>
-      <c r="H54" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="I54" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="J54" s="8" t="inlineStr">
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
@@ -3196,96 +3196,96 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="B59" s="8" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>16.06.2026</t>
         </is>
       </c>
-      <c r="C59" s="8" t="n">
+      <c r="C59" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D59" s="9" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>Argentinien - Algerien</t>
         </is>
       </c>
-      <c r="E59" s="9" t="inlineStr">
+      <c r="E59" s="5" t="inlineStr">
         <is>
           <t>Argentinien</t>
         </is>
       </c>
-      <c r="F59" s="9" t="inlineStr">
+      <c r="F59" s="5" t="inlineStr">
         <is>
           <t>Argentinien (1:0)</t>
         </is>
       </c>
-      <c r="G59" s="10" t="n">
+      <c r="G59" s="6" t="n">
         <v>0.72</v>
       </c>
-      <c r="H59" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="I59" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="J59" s="8" t="inlineStr">
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>16.06.2026</t>
         </is>
       </c>
-      <c r="C60" s="8" t="n">
+      <c r="C60" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D60" s="9" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>Österreich - Jordanien</t>
         </is>
       </c>
-      <c r="E60" s="9" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>Österreich</t>
         </is>
       </c>
-      <c r="F60" s="9" t="inlineStr">
+      <c r="F60" s="5" t="inlineStr">
         <is>
           <t>Österreich (1:0)</t>
         </is>
       </c>
-      <c r="G60" s="10" t="n">
+      <c r="G60" s="6" t="n">
         <v>0.68</v>
       </c>
-      <c r="H60" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="I60" s="8" t="inlineStr">
-        <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="J60" s="8" t="inlineStr">
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="I60" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
         <is>
           <t>2:0</t>
         </is>
@@ -4798,7 +4798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4819,7 +4819,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Sieger korrekt: 6/11 (~55 %) · Halbzeit-Führung korrekt: 6/11 (~55 %) · Exaktes Ergebnis: 2/11 (~18 %)</t>
+          <t>Sieger korrekt: 10/19 (~53 %) · Halbzeit-Führung korrekt: 6/13 (~46 %) · Exaktes Ergebnis: 2/19 (~11 %)</t>
         </is>
       </c>
     </row>
@@ -5239,8 +5239,264 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>15.06.</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Belgien - Ägypten</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Belgien 2:1</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>15.06.</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Iran - Neuseeland</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Iran 2:0</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>15.06.</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Spanien - Kap Verde</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Spanien 3:0</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>15.06.</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Saudi-Arabien - Uruguay</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Uruguay 0:2</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>16.06.</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Frankreich - Senegal</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Frankreich 2:1</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>16.06.</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Irak - Norwegen</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Norwegen 0:2</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>16.06.</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Argentinien - Algerien</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Argentinien 2:0</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>16.06.</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Österreich - Jordanien</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Österreich 2:0</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F16"/>
+  <autoFilter ref="A4:F24"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>